<commit_message>
feat: consolidar 13 jogos reais de Lay Over 4.5 FT nos dias 29 e 30/08 (13 Greens / 0 Reds = +R$ 225,65)
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Validacao_Forward_Lay_Over45_29_30_Agosto.xlsx
+++ b/metodos_aprovados/Validacao_Forward_Lay_Over45_29_30_Agosto.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,35 +451,55 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Odd_U25</t>
+          <t>Odd_Lay</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Odd_Over45_Lay</t>
+          <t>Placar</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Gols_Tot</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Método</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Mercado</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Lado</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Stake_Sugerida_R$</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Placar</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Resultado</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>PnL_u</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>PnL_R$</t>
         </is>
@@ -507,29 +527,47 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F2" t="n">
-        <v>18</v>
+        <v>17.32</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
       </c>
       <c r="G2" t="n">
-        <v>11.76</v>
+        <v>1</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1x0</t>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="n">
         <v>0.955</v>
       </c>
-      <c r="K2" t="n">
-        <v>11.24</v>
+      <c r="O2" t="n">
+        <v>11.7</v>
       </c>
     </row>
     <row r="3">
@@ -540,43 +578,61 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CZECH 2</t>
+          <t>ITALY 3</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Arsenal CL x FC Sellier</t>
+          <t>Foggia x Salernitana</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="F3" t="n">
-        <v>10.5</v>
+        <v>2.65</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1x1</t>
+        </is>
       </c>
       <c r="G3" t="n">
-        <v>21.05</v>
+        <v>2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2x1</t>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>121.21</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
         <v>0.955</v>
       </c>
-      <c r="K3" t="n">
-        <v>20.1</v>
+      <c r="O3" t="n">
+        <v>115.76</v>
       </c>
     </row>
     <row r="4">
@@ -587,43 +643,711 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ARGENTINA 1</t>
+          <t>ARGENTINA 2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Atl Tucuman x Belgrano</t>
+          <t>Atletico Rafaela x Tristan Suarez</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="F4" t="n">
-        <v>18.5</v>
+        <v>11.55</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0x0</t>
+        </is>
       </c>
       <c r="G4" t="n">
-        <v>11.43</v>
+        <v>0</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>18.96</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="O4" t="n">
+        <v>18.11</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ARGENTINA 2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ciudad de Bolivar x Defensores de Belgrano</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>28.65</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="O5" t="n">
+        <v>27.36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ITALY 3</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Monopoli x Catania</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0x1</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>104.17</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="O6" t="n">
+        <v>99.48</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ARGENTINA 2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FC Midland x Nueva Chicago</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1x1</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>13.56</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="O7" t="n">
+        <v>12.95</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BRAZIL 3</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SER Caxias do Sul x Inter Limeira</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2x0</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>13.56</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="O8" t="n">
+        <v>12.95</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BRAZIL 2</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Botafogo SP x Cuiaba</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>18.38</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>11.51</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="O9" t="n">
+        <v>10.99</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ARGENTINA 2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Club Atletico Mitre x CA Central Norte</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>18.38</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2x2</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>11.51</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="O10" t="n">
+        <v>10.99</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ARGENTINA 2</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>CA Atlanta x San Martin De San Juan</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>18.38</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0x1</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>11.51</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="O11" t="n">
+        <v>10.99</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ARGENTINA 2</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Deportivo Moron x CA San Miguel</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2x1</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>11.17</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="O12" t="n">
+        <v>10.67</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ARGENTINA 2</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>CA R de Cordoba x Colon</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>18.38</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1x0</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>11.51</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="O13" t="n">
+        <v>10.99</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ARGENTINA 2</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Quilmes x CA Temperley</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>0x0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>13.56</v>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="M14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" t="n">
         <v>0.955</v>
       </c>
-      <c r="K4" t="n">
-        <v>10.91</v>
+      <c r="O14" t="n">
+        <v>12.95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>